<commit_message>
Add more Recommend Data - Chinese, French
</commit_message>
<xml_diff>
--- a/public/data/speedvoca-free-data.xlsx
+++ b/public/data/speedvoca-free-data.xlsx
@@ -3,11 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Daily Life Conversation" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Restaurant &amp; Shopping" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Travel &amp; Transportation" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Social &amp; Small Talk" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Work  Office Communication" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="English Daily Conversation" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Chinese Daily Conversation" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="French Daily Conversation" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="English Restaurant &amp; Shopping" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="English Travel &amp; Transportation" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="English Social &amp; Small Talk" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="English Work  Office Communicat" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -15,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="393">
   <si>
     <t>sentence</t>
   </si>
@@ -201,6 +203,282 @@
   </si>
   <si>
     <t>저는 평화로운 순간을 좋아해요.</t>
+  </si>
+  <si>
+    <t>你好吗？</t>
+  </si>
+  <si>
+    <t>잘 지내?</t>
+  </si>
+  <si>
+    <t>我很好</t>
+  </si>
+  <si>
+    <t>나 잘 지내</t>
+  </si>
+  <si>
+    <t>我在路上</t>
+  </si>
+  <si>
+    <t>가는 중이야</t>
+  </si>
+  <si>
+    <t>你在做什么？</t>
+  </si>
+  <si>
+    <t>뭐 하고 있어?</t>
+  </si>
+  <si>
+    <t>我很忙</t>
+  </si>
+  <si>
+    <t>나 바빠</t>
+  </si>
+  <si>
+    <t>等我一下</t>
+  </si>
+  <si>
+    <t>나 좀 기다려</t>
+  </si>
+  <si>
+    <t>我们明天见</t>
+  </si>
+  <si>
+    <t>내일 보자</t>
+  </si>
+  <si>
+    <t>几点？</t>
+  </si>
+  <si>
+    <t>몇 시에?</t>
+  </si>
+  <si>
+    <t>我迟到了</t>
+  </si>
+  <si>
+    <t>나 늦었어</t>
+  </si>
+  <si>
+    <t>快点</t>
+  </si>
+  <si>
+    <t>서둘러</t>
+  </si>
+  <si>
+    <t>我明白了</t>
+  </si>
+  <si>
+    <t>이해했어</t>
+  </si>
+  <si>
+    <t>我不明白</t>
+  </si>
+  <si>
+    <t>이해 못 했어</t>
+  </si>
+  <si>
+    <t>请再说一遍</t>
+  </si>
+  <si>
+    <t>다시 말해줘</t>
+  </si>
+  <si>
+    <t>可以</t>
+  </si>
+  <si>
+    <t>좋아 / 괜찮아</t>
+  </si>
+  <si>
+    <t>没问题</t>
+  </si>
+  <si>
+    <t>문제 없어</t>
+  </si>
+  <si>
+    <t>非常感谢</t>
+  </si>
+  <si>
+    <t>정말 고마워</t>
+  </si>
+  <si>
+    <t>不客气</t>
+  </si>
+  <si>
+    <t>천만에</t>
+  </si>
+  <si>
+    <t>不好意思</t>
+  </si>
+  <si>
+    <t>미안해 / 실례해</t>
+  </si>
+  <si>
+    <t>好的</t>
+  </si>
+  <si>
+    <t>오케이</t>
+  </si>
+  <si>
+    <t>我们走吧</t>
+  </si>
+  <si>
+    <t>갈까?</t>
+  </si>
+  <si>
+    <t>我马上到</t>
+  </si>
+  <si>
+    <t>지금 가는 중이야</t>
+  </si>
+  <si>
+    <t>我累了</t>
+  </si>
+  <si>
+    <t>나 피곤해</t>
+  </si>
+  <si>
+    <t>我饿了</t>
+  </si>
+  <si>
+    <t>배고파</t>
+  </si>
+  <si>
+    <t>我渴了</t>
+  </si>
+  <si>
+    <t>목말라</t>
+  </si>
+  <si>
+    <t>我们去吃饭吧</t>
+  </si>
+  <si>
+    <t>밥 먹으러 가자</t>
+  </si>
+  <si>
+    <t>你想要什么？</t>
+  </si>
+  <si>
+    <t>뭐 원해?</t>
+  </si>
+  <si>
+    <t>远吗？</t>
+  </si>
+  <si>
+    <t>멀어?</t>
+  </si>
+  <si>
+    <t>很近</t>
+  </si>
+  <si>
+    <t>가까워</t>
+  </si>
+  <si>
+    <t>我同意</t>
+  </si>
+  <si>
+    <t>동의해</t>
+  </si>
+  <si>
+    <t>以后再说</t>
+  </si>
+  <si>
+    <t>나중에 보자</t>
+  </si>
+  <si>
+    <t>Comment ça va ?</t>
+  </si>
+  <si>
+    <t>Ça va bien</t>
+  </si>
+  <si>
+    <t>잘 지내</t>
+  </si>
+  <si>
+    <t>Je suis en route</t>
+  </si>
+  <si>
+    <t>Qu’est-ce que tu fais ?</t>
+  </si>
+  <si>
+    <t>Je suis occupé</t>
+  </si>
+  <si>
+    <t>Attends-moi</t>
+  </si>
+  <si>
+    <t>On se voit demain</t>
+  </si>
+  <si>
+    <t>À quelle heure ?</t>
+  </si>
+  <si>
+    <t>Je suis en retard</t>
+  </si>
+  <si>
+    <t>나 늦고 있어</t>
+  </si>
+  <si>
+    <t>Dépêche-toi</t>
+  </si>
+  <si>
+    <t>Je comprends</t>
+  </si>
+  <si>
+    <t>Je ne comprends pas</t>
+  </si>
+  <si>
+    <t>Répète s’il te plaît</t>
+  </si>
+  <si>
+    <t>C’est bon</t>
+  </si>
+  <si>
+    <t>Pas de problème</t>
+  </si>
+  <si>
+    <t>Merci beaucoup</t>
+  </si>
+  <si>
+    <t>De rien</t>
+  </si>
+  <si>
+    <t>Excuse-moi</t>
+  </si>
+  <si>
+    <t>Ça marche</t>
+  </si>
+  <si>
+    <t>On y va ?</t>
+  </si>
+  <si>
+    <t>J’arrive</t>
+  </si>
+  <si>
+    <t>Je suis fatigué</t>
+  </si>
+  <si>
+    <t>J’ai faim</t>
+  </si>
+  <si>
+    <t>J’ai soif</t>
+  </si>
+  <si>
+    <t>Allons manger</t>
+  </si>
+  <si>
+    <t>Tu veux quoi ?</t>
+  </si>
+  <si>
+    <t>C’est loin ?</t>
+  </si>
+  <si>
+    <t>C’est près</t>
+  </si>
+  <si>
+    <t>Je suis d’accord</t>
+  </si>
+  <si>
+    <t>On verra</t>
   </si>
   <si>
     <t>Can I see the menu?</t>
@@ -991,6 +1269,14 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1463,6 +1749,532 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="11.0"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="17.63"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
     <col customWidth="1" min="1" max="1" width="25.38"/>
     <col customWidth="1" min="2" max="2" width="23.0"/>
   </cols>
@@ -1477,242 +2289,242 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>154</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>63</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>64</v>
+        <v>156</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>65</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>66</v>
+        <v>158</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>67</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>68</v>
+        <v>160</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>69</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>70</v>
+        <v>162</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>71</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>73</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>74</v>
+        <v>166</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>75</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>76</v>
+        <v>168</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>77</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>78</v>
+        <v>170</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>79</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>80</v>
+        <v>172</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>81</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>82</v>
+        <v>174</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>83</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>84</v>
+        <v>176</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>85</v>
+        <v>177</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>86</v>
+        <v>178</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>87</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>88</v>
+        <v>180</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>89</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>90</v>
+        <v>182</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>91</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>92</v>
+        <v>184</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>93</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>94</v>
+        <v>186</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>95</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>96</v>
+        <v>188</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>97</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>98</v>
+        <v>190</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>99</v>
+        <v>191</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>100</v>
+        <v>192</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>101</v>
+        <v>193</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>102</v>
+        <v>194</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>103</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>104</v>
+        <v>196</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>105</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>106</v>
+        <v>198</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>107</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>108</v>
+        <v>200</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>109</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>110</v>
+        <v>202</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>111</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>112</v>
+        <v>204</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>113</v>
+        <v>205</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>114</v>
+        <v>206</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>115</v>
+        <v>207</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>116</v>
+        <v>208</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>117</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>118</v>
+        <v>210</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>119</v>
+        <v>211</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>120</v>
+        <v>212</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>121</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -1720,7 +2532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1741,242 +2553,242 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>122</v>
+        <v>214</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>124</v>
+        <v>216</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>125</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>126</v>
+        <v>218</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>127</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>128</v>
+        <v>220</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>129</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>130</v>
+        <v>222</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>131</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>132</v>
+        <v>224</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>133</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>134</v>
+        <v>226</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>135</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>136</v>
+        <v>228</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>137</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>138</v>
+        <v>230</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>139</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>140</v>
+        <v>232</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>141</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>142</v>
+        <v>234</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>143</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>144</v>
+        <v>236</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>145</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>146</v>
+        <v>238</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>147</v>
+        <v>239</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>148</v>
+        <v>240</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>149</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>150</v>
+        <v>242</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>151</v>
+        <v>243</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>152</v>
+        <v>244</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>153</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>154</v>
+        <v>246</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>155</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>156</v>
+        <v>248</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>157</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>158</v>
+        <v>250</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>159</v>
+        <v>251</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>160</v>
+        <v>252</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>161</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>162</v>
+        <v>254</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>163</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>164</v>
+        <v>256</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>165</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>166</v>
+        <v>258</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>167</v>
+        <v>259</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>168</v>
+        <v>260</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>169</v>
+        <v>261</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>170</v>
+        <v>262</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>79</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>171</v>
+        <v>263</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>172</v>
+        <v>264</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>173</v>
+        <v>265</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>174</v>
+        <v>266</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>175</v>
+        <v>267</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>176</v>
+        <v>268</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>177</v>
+        <v>269</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>178</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>179</v>
+        <v>271</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>180</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -1984,7 +2796,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2005,242 +2817,242 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>181</v>
+        <v>273</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>182</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>183</v>
+        <v>275</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>184</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>185</v>
+        <v>277</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>186</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>187</v>
+        <v>279</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>188</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>189</v>
+        <v>281</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>190</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>191</v>
+        <v>283</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>192</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>193</v>
+        <v>285</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>194</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>195</v>
+        <v>287</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>196</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>197</v>
+        <v>289</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>198</v>
+        <v>290</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>199</v>
+        <v>291</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>200</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>201</v>
+        <v>293</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>202</v>
+        <v>294</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>203</v>
+        <v>295</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>204</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>205</v>
+        <v>297</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>206</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>207</v>
+        <v>299</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>208</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>209</v>
+        <v>301</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>210</v>
+        <v>302</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>211</v>
+        <v>303</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>212</v>
+        <v>304</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>213</v>
+        <v>305</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>214</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>215</v>
+        <v>307</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>216</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>217</v>
+        <v>309</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>218</v>
+        <v>310</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>219</v>
+        <v>311</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>220</v>
+        <v>312</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>221</v>
+        <v>313</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>222</v>
+        <v>314</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>223</v>
+        <v>315</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>224</v>
+        <v>316</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>225</v>
+        <v>317</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>226</v>
+        <v>318</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>227</v>
+        <v>319</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>228</v>
+        <v>320</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>229</v>
+        <v>321</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>230</v>
+        <v>322</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>231</v>
+        <v>323</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>232</v>
+        <v>324</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>233</v>
+        <v>325</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>234</v>
+        <v>326</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>235</v>
+        <v>327</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>236</v>
+        <v>328</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>237</v>
+        <v>329</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>238</v>
+        <v>330</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>239</v>
+        <v>331</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>240</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -2248,7 +3060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2269,242 +3081,242 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>241</v>
+        <v>333</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>242</v>
+        <v>334</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>243</v>
+        <v>335</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>244</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>245</v>
+        <v>337</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>246</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>247</v>
+        <v>339</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>248</v>
+        <v>340</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>249</v>
+        <v>341</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>250</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>251</v>
+        <v>343</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>252</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>253</v>
+        <v>345</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>254</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>255</v>
+        <v>347</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>256</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>257</v>
+        <v>349</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>258</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>259</v>
+        <v>351</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>260</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>261</v>
+        <v>353</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>262</v>
+        <v>354</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>263</v>
+        <v>355</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>264</v>
+        <v>356</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>265</v>
+        <v>357</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>266</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>267</v>
+        <v>359</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>268</v>
+        <v>360</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>269</v>
+        <v>361</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>270</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>271</v>
+        <v>363</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>272</v>
+        <v>364</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>273</v>
+        <v>365</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>274</v>
+        <v>366</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>275</v>
+        <v>367</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>276</v>
+        <v>368</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>277</v>
+        <v>369</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>278</v>
+        <v>370</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>279</v>
+        <v>371</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>280</v>
+        <v>372</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>281</v>
+        <v>373</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>282</v>
+        <v>374</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>283</v>
+        <v>375</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>284</v>
+        <v>376</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>285</v>
+        <v>377</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>286</v>
+        <v>378</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>287</v>
+        <v>379</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>288</v>
+        <v>380</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>289</v>
+        <v>381</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>290</v>
+        <v>382</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>291</v>
+        <v>383</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>292</v>
+        <v>384</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>293</v>
+        <v>385</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>294</v>
+        <v>386</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>295</v>
+        <v>387</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>296</v>
+        <v>388</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>297</v>
+        <v>389</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>298</v>
+        <v>390</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>299</v>
+        <v>391</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>300</v>
+        <v>392</v>
       </c>
     </row>
   </sheetData>

</xml_diff>